<commit_message>
Analysis Add-ins workbook: set calculation to automatic
It was saved in manual mode, so students who opened it first got manual
calculation and What-If scenario summaries showed the same values.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/6_Advanced_Data_Analysis/1_Analysis_Add-ins.xlsx
+++ b/6_Advanced_Data_Analysis/1_Analysis_Add-ins.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30618"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Developer\_Courses\Excel\Excel_Data_Analytics_Course\6_Advanced_Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C309F530-9477-46F8-BC41-B3020D3E60A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFBEB8D-B6C4-4401-BFA6-99DF5CA2F903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="18336" windowHeight="10428" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="18240" windowHeight="10344" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Forecast_Original" sheetId="7" r:id="rId1"/>
@@ -63,7 +63,7 @@
     <definedName name="Year3">'What-If_Analysis'!$C$12</definedName>
     <definedName name="Year4">'What-If_Analysis'!$C$13</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="manual"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -7462,6 +7462,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7469,7 +7470,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>

</xml_diff>